<commit_message>
Flip click Feature added
</commit_message>
<xml_diff>
--- a/projectCharter_schedule/Sbraynen_Project Schedule.xlsx
+++ b/projectCharter_schedule/Sbraynen_Project Schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0112e2c07da1ee9a/Desktop/WINTER 2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="154" documentId="8_{9B65AEB0-4F86-4149-8026-09A7893626D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53D6CC4D-B071-4106-92BF-4FFEFCA4C34E}"/>
+  <xr:revisionPtr revIDLastSave="159" documentId="8_{9B65AEB0-4F86-4149-8026-09A7893626D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18139D0F-8F52-4746-B092-B25881EF2C04}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
   <si>
     <t>Start Date</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>Active</t>
-  </si>
-  <si>
-    <t>Upcoming</t>
   </si>
   <si>
     <t>Meet The Artist</t>
@@ -145,7 +142,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -170,14 +167,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="13">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -325,11 +316,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -369,6 +373,27 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="24"/>
     </xf>
@@ -378,35 +403,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="24"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -423,6 +421,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -634,25 +636,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="24.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="17"/>
+      <c r="A1" s="22" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="24"/>
     </row>
     <row r="2" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="18" t="s">
+      <c r="D2" s="15" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="10" t="s">
@@ -661,7 +663,7 @@
     </row>
     <row r="3" spans="1:5" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="5">
         <v>46050</v>
@@ -669,16 +671,16 @@
       <c r="C3" s="11">
         <v>46050</v>
       </c>
-      <c r="D3" s="25" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="19" t="s">
+      <c r="D3" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="16" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="21.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="5">
         <v>46050</v>
@@ -686,16 +688,16 @@
       <c r="C4" s="12">
         <v>46053</v>
       </c>
-      <c r="D4" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="19" t="s">
+      <c r="D4" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="16" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="36.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" s="5">
         <v>46051</v>
@@ -703,16 +705,16 @@
       <c r="C5" s="12">
         <v>46055</v>
       </c>
-      <c r="D5" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="20" t="s">
-        <v>16</v>
+      <c r="D5" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="6">
         <v>46071</v>
@@ -720,16 +722,16 @@
       <c r="C6" s="13">
         <v>46098</v>
       </c>
-      <c r="D6" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>5</v>
+      <c r="D6" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="30.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B7" s="5">
         <v>46081</v>
@@ -737,16 +739,16 @@
       <c r="C7" s="12">
         <v>46099</v>
       </c>
-      <c r="D7" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="24.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D7" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="24.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="5">
         <v>46082</v>
@@ -754,16 +756,16 @@
       <c r="C8" s="12">
         <v>46099</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="23" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="E8" s="23" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="23" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="4" t="s">
-        <v>21</v>
       </c>
       <c r="B9" s="7">
         <v>46100</v>
@@ -771,11 +773,11 @@
       <c r="C9" s="14">
         <v>46101</v>
       </c>
-      <c r="D9" s="27" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>6</v>
+      <c r="D9" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>